<commit_message>
Pivot targeting to Dev Agency leads
</commit_message>
<xml_diff>
--- a/creator-leads.xlsx
+++ b/creator-leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="109">
   <si>
     <t>Creator Name</t>
   </si>
@@ -49,6 +49,114 @@
     <t>Tech Stack</t>
   </si>
   <si>
+    <t>Sonny Sangha</t>
+  </si>
+  <si>
+    <t>https://youtube.com/@sonnysangha</t>
+  </si>
+  <si>
+    <t>https://www.papareact.com/course</t>
+  </si>
+  <si>
+    <t>GB</t>
+  </si>
+  <si>
+    <t>2026-07-20</t>
+  </si>
+  <si>
+    <t>styles@1.4.0</t>
+  </si>
+  <si>
+    <t>Courses, SaaS, Membership, Digital products, Coaching</t>
+  </si>
+  <si>
+    <t>AI chatbot, Custom coding challenge platform, Advanced analytics dashboard, Membership portal, Internal admin panel</t>
+  </si>
+  <si>
+    <t>As a fellow developer and admirer of your work helping aspiring coders through PAPA React and "Zero to Full Stack Hero," I'm curious if you've ever considered custom software to further enhance your student's learning experience or streamline your operations beyond Kajabi's capabilities.</t>
+  </si>
+  <si>
+    <t>Kajabi</t>
+  </si>
+  <si>
+    <t>This Week in Startups</t>
+  </si>
+  <si>
+    <t>https://youtube.com/@startups</t>
+  </si>
+  <si>
+    <t>https://rb.gy/v19fcp</t>
+  </si>
+  <si>
+    <t>US</t>
+  </si>
+  <si>
+    <t>2026-07-17</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Courses, Templates, SaaS, Newsletter, Digital products</t>
+  </si>
+  <si>
+    <t>Sponsorship Dashboard, Internal Admin Panel, Custom Course Platform, AI Chatbot, CRM</t>
+  </si>
+  <si>
+    <t>Jason, I've been following This Week in Startups for years and am consistently impressed by your ability to not only cover the startup world but also build a thriving digital products business; I'm curious how you manage the diverse offerings from courses to SaaS.</t>
+  </si>
+  <si>
+    <t>Shopify</t>
+  </si>
+  <si>
+    <t>ATO Automation</t>
+  </si>
+  <si>
+    <t>https://youtube.com/@atocom-automation</t>
+  </si>
+  <si>
+    <t>https://www.ato.com/</t>
+  </si>
+  <si>
+    <t>2026-07-16</t>
+  </si>
+  <si>
+    <t>service@ato.com</t>
+  </si>
+  <si>
+    <t>Newsletter</t>
+  </si>
+  <si>
+    <t>CRM, AI chatbot, Internal admin panel, Analytics dashboard, Supplier management portal, Email automation</t>
+  </si>
+  <si>
+    <t>Your direct-to-consumer model for industrial automation components is impressive, and I'm curious how you currently manage the expert support you offer for choosing, wiring, and commissioning these complex products.</t>
+  </si>
+  <si>
+    <t>Coding Blocks</t>
+  </si>
+  <si>
+    <t>https://youtube.com/@codingblocksindia</t>
+  </si>
+  <si>
+    <t>https://codingblocks.com/index.html</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>kamna.saroha@codingblocks.com</t>
+  </si>
+  <si>
+    <t>Courses, SaaS, Membership, Digital products, Templates</t>
+  </si>
+  <si>
+    <t>Course platform, Membership portal, Analytics dashboard, Internal admin panel, AI chatbot, CRM, Email automation</t>
+  </si>
+  <si>
+    <t>I was impressed by Coding Blocks' mission to create skilled software engineers and bridge the industry skill gap through practical training, and I believe custom software could further enhance your student experience and operational efficiency.</t>
+  </si>
+  <si>
     <t>Smart Programming</t>
   </si>
   <si>
@@ -58,12 +166,6 @@
     <t>https://www.smartprogramming.in</t>
   </si>
   <si>
-    <t>IN</t>
-  </si>
-  <si>
-    <t>2026-07-20</t>
-  </si>
-  <si>
     <t>bootstrap@5.0.2</t>
   </si>
   <si>
@@ -76,9 +178,6 @@
     <t>I was impressed by Smart Programming's comprehensive offerings in online programming training and project development, especially across such a wide range of technologies.</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>Rei丨暮らしとNotion。</t>
   </si>
   <si>
@@ -106,7 +205,25 @@
     <t>Rei-san, seeing your success as a Notion official ambassador and the impact of your 'Notion Lifehacks' book, I was curious if you've ever considered custom software to further enhance your template and membership offerings for your dedicated community.</t>
   </si>
   <si>
-    <t>Shopify</t>
+    <t>Paritosh Sharma - Shunya AI</t>
+  </si>
+  <si>
+    <t>https://youtube.com/@paritosh-sharma-shunyaai</t>
+  </si>
+  <si>
+    <t>https://join.shunyaai.com/new-courses/99-ai-foundation-for-students</t>
+  </si>
+  <si>
+    <t>wght@100..900</t>
+  </si>
+  <si>
+    <t>Courses</t>
+  </si>
+  <si>
+    <t>Custom Course Platform, AI Chatbot, Analytics Dashboard, CRM, Automated Assessment System</t>
+  </si>
+  <si>
+    <t>I was really impressed to learn about Shunya AI's mission to empower students and professionals in AI, and I'm curious if you've ever considered how custom software could further enhance your leading training programs.</t>
   </si>
   <si>
     <t>Saad Rashid - YouTube Automation</t>
@@ -121,9 +238,6 @@
     <t>PK</t>
   </si>
   <si>
-    <t>2026-07-17</t>
-  </si>
-  <si>
     <t>Digital products, Templates, Membership</t>
   </si>
   <si>
@@ -133,6 +247,81 @@
     <t>Saad, I'm impressed by your expertise in helping creators build successful faceless YouTube channels, and I'm curious how a custom platform could streamline your course delivery and student management.</t>
   </si>
   <si>
+    <t>AI動画ラボコイコイ</t>
+  </si>
+  <si>
+    <t>https://youtube.com/@ailabokoikoi</t>
+  </si>
+  <si>
+    <t>https://note.com/ai_labo_koikoi/n/n3939c2d25920</t>
+  </si>
+  <si>
+    <t>2026-07-15</t>
+  </si>
+  <si>
+    <t>Membership, Digital products</t>
+  </si>
+  <si>
+    <t>Membership portal, Course platform, AI tool integration, Analytics dashboard, Email automation</t>
+  </si>
+  <si>
+    <t>Your unique approach to creating and teaching others how to make AI-generated 'grandma' YouTuber videos is truly innovative, and I'm curious if you've ever considered custom software to enhance your membership offerings or streamline your content creation process.</t>
+  </si>
+  <si>
+    <t>Makes It With AI</t>
+  </si>
+  <si>
+    <t>https://youtube.com/@makesitwithai</t>
+  </si>
+  <si>
+    <t>https://bit.ly/Canva30DayFREETrial</t>
+  </si>
+  <si>
+    <t>2026-07-19</t>
+  </si>
+  <si>
+    <t>Affiliate Dashboard, Content Management System, AI Chatbot, Analytics Dashboard, Membership Portal</t>
+  </si>
+  <si>
+    <t>I'm really impressed with how you break down complex AI and Canva video creation into actionable steps with your 'Screen-To-Create Method' – have you ever considered how custom software could help you scale your tutorial production or better track your affiliate success?</t>
+  </si>
+  <si>
+    <t>Productive Setups</t>
+  </si>
+  <si>
+    <t>https://youtube.com/@productivesetups</t>
+  </si>
+  <si>
+    <t>https://productivesetups.gumroad.com/</t>
+  </si>
+  <si>
+    <t>2026-07-14</t>
+  </si>
+  <si>
+    <t>Digital product storefront, Email automation, Analytics dashboard</t>
+  </si>
+  <si>
+    <t>I've been enjoying your Productive Setups content and noticed your Gumroad link; I'm curious if you've considered custom tools to help launch and manage your digital products more effectively.</t>
+  </si>
+  <si>
+    <t>Coding2GO</t>
+  </si>
+  <si>
+    <t>https://youtube.com/@coding2go</t>
+  </si>
+  <si>
+    <t>https://coding2go.com)</t>
+  </si>
+  <si>
+    <t>2026-07-12</t>
+  </si>
+  <si>
+    <t>Course platform, Membership portal, Sponsorship dashboard, Interactive coding environment, Internal admin panel</t>
+  </si>
+  <si>
+    <t>Your mission to teach aspiring developers through fast-paced tutorials and Udemy courses is fantastic; I was thinking about how a custom course platform could help you offer even more structured learning directly on coding2go.com.</t>
+  </si>
+  <si>
     <t>Learn with Sumit - LWS - Bangladesh</t>
   </si>
   <si>
@@ -145,56 +334,17 @@
     <t>BD</t>
   </si>
   <si>
-    <t>2026-07-15</t>
-  </si>
-  <si>
     <t>Course platform, Membership portal, AI chatbot, Analytics dashboard, Internal admin panel</t>
   </si>
   <si>
     <t>I've been following your excellent work teaching web development, especially your focus on AI for JavaScript and backend developers in Bangla, and I believe custom software could significantly enhance your educational platform and student experience.</t>
-  </si>
-  <si>
-    <t>Productive Setups</t>
-  </si>
-  <si>
-    <t>https://youtube.com/@productivesetups</t>
-  </si>
-  <si>
-    <t>https://productivesetups.gumroad.com/</t>
-  </si>
-  <si>
-    <t>2026-07-14</t>
-  </si>
-  <si>
-    <t>Digital product storefront, Email automation, Analytics dashboard</t>
-  </si>
-  <si>
-    <t>I've been enjoying your Productive Setups content and noticed your Gumroad link; I'm curious if you've considered custom tools to help launch and manage your digital products more effectively.</t>
-  </si>
-  <si>
-    <t>Coding2GO</t>
-  </si>
-  <si>
-    <t>https://youtube.com/@coding2go</t>
-  </si>
-  <si>
-    <t>https://coding2go.com)</t>
-  </si>
-  <si>
-    <t>2026-07-12</t>
-  </si>
-  <si>
-    <t>Course platform, Membership portal, Sponsorship dashboard, Interactive coding environment, Internal admin panel</t>
-  </si>
-  <si>
-    <t>Your mission to teach aspiring developers through fast-paced tutorials and Udemy courses is fantastic; I was thinking about how a custom course platform could help you offer even more structured learning directly on coding2go.com.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -209,13 +359,22 @@
       <u/>
       <color rgb="0563C1"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF006100"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD4EDC9"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -230,9 +389,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -573,7 +735,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -627,78 +789,78 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E2">
-        <v>316000</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="E2" s="2">
+        <v>435000</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I2">
-        <v>75</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="I2" s="4">
+        <v>100</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E3">
-        <v>51300</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="E3" s="2">
+        <v>352000</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="G3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I3">
-        <v>55</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="I3" s="4">
+        <v>85</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="2" t="s">
         <v>31</v>
       </c>
     </row>
@@ -706,29 +868,29 @@
       <c r="A4" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="5" t="s">
         <v>34</v>
       </c>
       <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4">
+        <v>80200</v>
+      </c>
+      <c r="F4" t="s">
         <v>35</v>
       </c>
-      <c r="E4">
-        <v>199000</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>36</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
       </c>
       <c r="H4" t="s">
         <v>37</v>
       </c>
       <c r="I4">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="J4" t="s">
         <v>38</v>
@@ -737,121 +899,387 @@
         <v>39</v>
       </c>
       <c r="L4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="5" t="s">
         <v>42</v>
       </c>
       <c r="D5" t="s">
         <v>43</v>
       </c>
       <c r="E5">
-        <v>190000</v>
+        <v>254000</v>
       </c>
       <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
         <v>44</v>
       </c>
-      <c r="G5" t="s">
-        <v>21</v>
-      </c>
       <c r="H5" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="I5">
-        <v>10</v>
+        <v>75</v>
       </c>
       <c r="J5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L5" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="B6" s="5" t="s">
         <v>49</v>
       </c>
+      <c r="C6" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="E6">
-        <v>49700</v>
+        <v>316000</v>
       </c>
       <c r="F6" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="I6">
-        <v>10</v>
+        <v>75</v>
       </c>
       <c r="J6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="K6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L6" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" s="2" t="s">
         <v>55</v>
       </c>
+      <c r="B7" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="E7">
+        <v>51300</v>
+      </c>
+      <c r="F7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" t="s">
+        <v>60</v>
+      </c>
+      <c r="H7" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7">
+        <v>55</v>
+      </c>
+      <c r="J7" t="s">
+        <v>62</v>
+      </c>
+      <c r="K7" t="s">
+        <v>63</v>
+      </c>
+      <c r="L7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8">
+        <v>36700</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
+        <v>67</v>
+      </c>
+      <c r="H8" t="s">
+        <v>68</v>
+      </c>
+      <c r="I8">
+        <v>45</v>
+      </c>
+      <c r="J8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K8" t="s">
+        <v>70</v>
+      </c>
+      <c r="L8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9">
+        <v>200000</v>
+      </c>
+      <c r="F9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" t="s">
+        <v>75</v>
+      </c>
+      <c r="I9">
+        <v>40</v>
+      </c>
+      <c r="J9" t="s">
+        <v>76</v>
+      </c>
+      <c r="K9" t="s">
+        <v>77</v>
+      </c>
+      <c r="L9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10">
+        <v>118000</v>
+      </c>
+      <c r="F10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" t="s">
+        <v>82</v>
+      </c>
+      <c r="I10">
+        <v>40</v>
+      </c>
+      <c r="J10" t="s">
+        <v>83</v>
+      </c>
+      <c r="K10" t="s">
+        <v>84</v>
+      </c>
+      <c r="L10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11">
+        <v>41200</v>
+      </c>
+      <c r="F11" t="s">
+        <v>88</v>
+      </c>
+      <c r="G11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I11">
+        <v>35</v>
+      </c>
+      <c r="J11" t="s">
+        <v>89</v>
+      </c>
+      <c r="K11" t="s">
+        <v>90</v>
+      </c>
+      <c r="L11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12">
+        <v>49700</v>
+      </c>
+      <c r="F12" t="s">
+        <v>94</v>
+      </c>
+      <c r="G12" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" t="s">
+        <v>27</v>
+      </c>
+      <c r="I12">
+        <v>10</v>
+      </c>
+      <c r="J12" t="s">
+        <v>95</v>
+      </c>
+      <c r="K12" t="s">
+        <v>96</v>
+      </c>
+      <c r="L12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13">
         <v>253000</v>
       </c>
-      <c r="F7" t="s">
-        <v>56</v>
-      </c>
-      <c r="G7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I7">
+      <c r="F13" t="s">
+        <v>100</v>
+      </c>
+      <c r="G13" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" t="s">
+        <v>27</v>
+      </c>
+      <c r="I13">
         <v>10</v>
       </c>
-      <c r="J7" t="s">
-        <v>57</v>
-      </c>
-      <c r="K7" t="s">
-        <v>58</v>
-      </c>
-      <c r="L7" t="s">
-        <v>21</v>
+      <c r="J13" t="s">
+        <v>101</v>
+      </c>
+      <c r="K13" t="s">
+        <v>102</v>
+      </c>
+      <c r="L13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" t="s">
+        <v>106</v>
+      </c>
+      <c r="E14">
+        <v>190000</v>
+      </c>
+      <c r="F14" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" t="s">
+        <v>27</v>
+      </c>
+      <c r="I14">
+        <v>10</v>
+      </c>
+      <c r="J14" t="s">
+        <v>107</v>
+      </c>
+      <c r="K14" t="s">
+        <v>108</v>
+      </c>
+      <c r="L14" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -869,6 +1297,20 @@
     <hyperlink ref="C6" r:id="rId10"/>
     <hyperlink ref="B7" r:id="rId11"/>
     <hyperlink ref="C7" r:id="rId12"/>
+    <hyperlink ref="B8" r:id="rId13"/>
+    <hyperlink ref="C8" r:id="rId14"/>
+    <hyperlink ref="B9" r:id="rId15"/>
+    <hyperlink ref="C9" r:id="rId16"/>
+    <hyperlink ref="B10" r:id="rId17"/>
+    <hyperlink ref="C10" r:id="rId18"/>
+    <hyperlink ref="B11" r:id="rId19"/>
+    <hyperlink ref="C11" r:id="rId20"/>
+    <hyperlink ref="B12" r:id="rId21"/>
+    <hyperlink ref="C12" r:id="rId22"/>
+    <hyperlink ref="B13" r:id="rId23"/>
+    <hyperlink ref="C13" r:id="rId24"/>
+    <hyperlink ref="B14" r:id="rId25"/>
+    <hyperlink ref="C14" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>